<commit_message>
docs(requirements): sync v1.2 decisions across sources
</commit_message>
<xml_diff>
--- a/Save_a_Life.xlsx
+++ b/Save_a_Life.xlsx
@@ -842,12 +842,12 @@
     <row r="22" ht="50" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Decisiones pendientes</t>
+          <t>Decisiones cerradas y pendientes</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Radio y ampliación por urgencia · significado de cantidad · estados exactos · intervalo post-donación y fuente clínica · precisión, retención y eliminación de ubicación · detalles operativos de Resend · validación legal aplicable en Perú.</t>
+          <t>Cerradas 2026-10-01: sin historial de ultima donacion ni filtro postdonacion (RF-PRO-05/RF-MAT-01); alta asistida 24 h y reemision sin reiniciar purga (AP-01); ocultar identidad tras confirmar a rechazar (AP-03); token de email 24 h (AP-05); invitacion/token vence con la necesidad (AP-09). Pendientes: operativa Resend/AP-02/AP-06/AP-08; resultados de carreras/AP-04; backups/AP-07; precision/retencion de ubicacion; revision legal en Peru.</t>
         </is>
       </c>
     </row>
@@ -1368,17 +1368,17 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Como donante quiero registrar la fecha de mi última donación.</t>
+          <t>La plataforma no solicita, acepta, almacena ni infiere fecha o historial de ultima donacion (RF-PRO-05).</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>W</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Rechaza fechas futuras; el bloqueo usa una política configurable, versionada y aprobada clínicamente; sin ella el sistema no inventa un intervalo ni afirma elegibilidad.</t>
+          <t>No existe campo de fecha/historial; rechazar mass assignment y no inferir bloqueos. Ver RF-PRO-05 y RF-MAT-01.</t>
         </is>
       </c>
     </row>
@@ -1611,17 +1611,17 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Como admin de hospital quiero excluir candidatos no disponibles o con bloqueo vigente.</t>
+          <t>Como admin de hospital quiero que la preseleccion excluya donantes no disponibles y use solo los filtros aprobados; no aplicar bloqueo postdonacion.</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Excluye no disponibles; el bloqueo solo se aplica con una política clínica aprobada y configurable; sin política no se ejecuta ese filtro ni se afirma elegibilidad.</t>
+          <t>Excluye cuentas inactivas, perfiles incompletos, no disponibles y ubicaciones invalidas/fuera del poligono; sin filtro por ultima donacion ni afirmacion de elegibilidad medica.</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>El donante gestiona únicamente su grupo sanguíneo declarado, ubicación, disponibilidad y fecha de última donación.</t>
+          <t>El donante gestiona grupo sanguineo declarado, ubicacion y disponibilidad; la plataforma no solicita, acepta, almacena ni infiere fecha/historial de ultima donacion (RF-PRO-05).</t>
         </is>
       </c>
     </row>
@@ -2206,7 +2206,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>El bloqueo post-donación solo se aplica con una regla configurable, versionada y aprobada por una fuente clínica competente; no se hardcodean intervalos.</t>
+          <t>El filtro postdonacion permanece desactivado; no se solicita ni infiere historial. La preseleccion solo aplica criterios academicos para datos sinteticos y no certifica elegibilidad medica (RF-MAT-01/RF-PRO-05).</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Matriz ABO/Rh, Haversine, disponibilidad, bloqueo configurable y orden estable</t>
+          <t>Matriz RBC academica, Haversine, cuenta activa/perfil completo, disponibilidad, ubicacion Lima, orden estable y cuotas; sin filtro postdonacion.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">

</xml_diff>